<commit_message>
fixed no current series
</commit_message>
<xml_diff>
--- a/database/series_setup.xlsx
+++ b/database/series_setup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="44">
   <si>
     <t>Name</t>
   </si>
@@ -39,79 +39,115 @@
     <t>SeriesName</t>
   </si>
   <si>
-    <t>Harrys Race Series #1 2026</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Current</t>
   </si>
   <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>Complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harrys Race SX </t>
-  </si>
-  <si>
-    <t>Harrys Race SZ</t>
-  </si>
-  <si>
-    <t>Harrys Race SX</t>
-  </si>
-  <si>
-    <t>Stage Uno</t>
-  </si>
-  <si>
-    <t>Stage Dos</t>
-  </si>
-  <si>
-    <t>Stage Tres</t>
-  </si>
-  <si>
-    <t>Stage Quatro</t>
-  </si>
-  <si>
-    <t>Stage Cinco</t>
-  </si>
-  <si>
-    <t>Stage Seis</t>
-  </si>
-  <si>
     <t>America/Toronto</t>
   </si>
   <si>
     <t>Local TZ</t>
   </si>
   <si>
-    <t>5c474c9b-cc47-4f65-8d5c-5a206475988c</t>
-  </si>
-  <si>
-    <t>c92abe92-7e93-40e3-9500-378cd792639f</t>
-  </si>
-  <si>
-    <t>Mungia | Spain</t>
-  </si>
-  <si>
-    <t>Sunset Ride from Calvi | Corsica</t>
-  </si>
-  <si>
     <t>EventId</t>
   </si>
   <si>
-    <t>d257a5e4-3b0e-4f3e-b0a7-084ad404df3e</t>
-  </si>
-  <si>
-    <t>Stage X</t>
-  </si>
-  <si>
-    <t>b02d01d1-d21e-4095-8788-878691be5de9</t>
-  </si>
-  <si>
-    <t>a880966a-1325-4a1d-882a-ece2dcbf9244</t>
+    <t>Harrys TT Series #1 Fall 2026</t>
+  </si>
+  <si>
+    <t>Bagnara C. to Cannitello over Scilla - Calabria</t>
+  </si>
+  <si>
+    <t>Arta to Playa de Muro | Mallorca</t>
+  </si>
+  <si>
+    <t>Antsampanimahazo | Madagascar</t>
+  </si>
+  <si>
+    <t>Stage 4. Madagascar</t>
+  </si>
+  <si>
+    <t>Stage 7. Mallorca</t>
+  </si>
+  <si>
+    <t>Kato Gouves to Herakleion | Crete</t>
+  </si>
+  <si>
+    <t>Stage 3. Crete</t>
+  </si>
+  <si>
+    <t>Dambula to Lion Rock on Road | Sri Lanka</t>
+  </si>
+  <si>
+    <t>Stage 6. Sri Lanka</t>
+  </si>
+  <si>
+    <t>Stage 5. Calabria</t>
+  </si>
+  <si>
+    <t>Lago di Garda North West | Italy</t>
+  </si>
+  <si>
+    <t>Stage 1. Lago di Garda</t>
+  </si>
+  <si>
+    <t>Stage 2. Porto</t>
+  </si>
+  <si>
+    <t>Porto | Portugal</t>
+  </si>
+  <si>
+    <t>Stage</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>Tu</t>
+  </si>
+  <si>
+    <t>We</t>
+  </si>
+  <si>
+    <t>Th</t>
+  </si>
+  <si>
+    <t>Time EST</t>
+  </si>
+  <si>
+    <t>Harrys TT Series Stage 1 - harrysracing.ca</t>
+  </si>
+  <si>
+    <t>Harrys TT Series Stage 2 - harrysracing.ca</t>
+  </si>
+  <si>
+    <t>Harrys TT Series Stage 3 - harrysracing.ca</t>
+  </si>
+  <si>
+    <t>Harrys TT Series Stage 4 - harrysracing.ca</t>
+  </si>
+  <si>
+    <t>Harrys TT Series Stage 5 - harrysracing.ca</t>
+  </si>
+  <si>
+    <t>Harrys TT Series Stage 6 - harrysracing.ca</t>
+  </si>
+  <si>
+    <t>9:30am</t>
+  </si>
+  <si>
+    <t>12:30PM</t>
+  </si>
+  <si>
+    <t>3:30PM</t>
+  </si>
+  <si>
+    <t>5:30PM</t>
   </si>
 </sst>
 </file>
@@ -158,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
@@ -169,6 +205,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,14 +518,14 @@
   <cols>
     <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -500,68 +540,36 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3">
-        <v>46235</v>
+        <v>46286</v>
       </c>
       <c r="D2" s="3">
-        <v>46283</v>
+        <v>46334</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="3">
-        <v>46235</v>
-      </c>
-      <c r="D3" s="3">
-        <v>46283</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3">
-        <v>46235</v>
-      </c>
-      <c r="D4" s="3">
-        <v>46283</v>
-      </c>
-      <c r="E4">
-        <v>7</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I9" s="4"/>
@@ -612,22 +620,22 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C2" s="3">
-        <v>46249</v>
+        <v>46286</v>
       </c>
       <c r="D2" s="3">
-        <v>46255</v>
+        <v>46290</v>
       </c>
       <c r="E2" s="6">
-        <v>96466</v>
+        <v>96854</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -636,47 +644,50 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3">
-        <v>46256</v>
+        <v>46293</v>
       </c>
       <c r="D3" s="3">
-        <v>46262</v>
+        <v>46297</v>
       </c>
       <c r="E3" s="6">
-        <v>251360</v>
+        <v>251103</v>
       </c>
       <c r="F3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C4" s="3">
-        <v>46263</v>
+        <v>46300</v>
       </c>
       <c r="D4" s="3">
-        <v>46269</v>
+        <v>46304</v>
       </c>
       <c r="E4" s="6">
-        <v>251436</v>
+        <v>96024</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3">
         <v>46270</v>
@@ -687,56 +698,68 @@
       <c r="E5" s="6">
         <v>96701</v>
       </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C6" s="3">
-        <v>46277</v>
+        <v>46307</v>
       </c>
       <c r="D6" s="3">
-        <v>46283</v>
+        <v>46311</v>
       </c>
       <c r="E6" s="6">
-        <v>96854</v>
+        <v>250261</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="3">
+        <v>46314</v>
+      </c>
+      <c r="D7" s="3">
+        <v>46318</v>
+      </c>
+      <c r="E7" s="6">
+        <v>97043</v>
+      </c>
+      <c r="F7" t="s">
         <v>20</v>
-      </c>
-      <c r="C7" s="3">
-        <v>46284</v>
-      </c>
-      <c r="D7" s="3">
-        <v>46290</v>
-      </c>
-      <c r="E7" s="6">
-        <v>251103</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="3">
+        <v>46321</v>
+      </c>
+      <c r="D8" s="3">
+        <v>46325</v>
+      </c>
+      <c r="E8" s="6">
+        <v>96479</v>
+      </c>
+      <c r="F8" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="3">
-        <v>46305</v>
-      </c>
-      <c r="D8" s="3">
-        <v>46252</v>
-      </c>
-      <c r="E8" s="6">
-        <v>96854</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -780,41 +803,1226 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="9"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>31</v>
+      <c r="E1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="8">
+        <v>46287</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="9">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="8">
+        <v>46287</v>
+      </c>
+      <c r="E3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="8">
+        <v>46287</v>
+      </c>
+      <c r="E4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="8">
+        <v>46287</v>
+      </c>
+      <c r="E5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B6" s="9">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="8">
+        <v>46288</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B7" s="9">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="8">
+        <v>46288</v>
+      </c>
+      <c r="E7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B8" s="9">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="8">
+        <v>46288</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B9" s="9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="8">
+        <v>46288</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="8">
+        <v>46289</v>
+      </c>
+      <c r="E10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="9">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="8">
+        <v>46289</v>
+      </c>
+      <c r="E11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="9">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="8">
+        <v>46289</v>
+      </c>
+      <c r="E12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="9">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="8">
+        <v>46289</v>
+      </c>
+      <c r="E13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="9">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="8">
+        <v>46294</v>
+      </c>
+      <c r="E14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="9">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="8">
+        <v>46294</v>
+      </c>
+      <c r="E15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="9">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="8">
+        <v>46294</v>
+      </c>
+      <c r="E16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="9">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="8">
+        <v>46294</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="9">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="9">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="9">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="9">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="9">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="8">
+        <v>46296</v>
+      </c>
+      <c r="E22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="9">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="8">
+        <v>46296</v>
+      </c>
+      <c r="E23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="9">
+        <v>2</v>
+      </c>
+      <c r="C24" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="8">
+        <v>46296</v>
+      </c>
+      <c r="E24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="9">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="8">
+        <v>46296</v>
+      </c>
+      <c r="E25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="9">
+        <v>3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D26" s="8">
+        <v>46301</v>
+      </c>
+      <c r="E26" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="9">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" s="8">
+        <v>46301</v>
+      </c>
+      <c r="E27" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="9">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="8">
+        <v>46301</v>
+      </c>
+      <c r="E28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="9">
+        <v>3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="8">
+        <v>46301</v>
+      </c>
+      <c r="E29" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B30" s="9">
+        <v>3</v>
+      </c>
+      <c r="C30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="8">
+        <v>46302</v>
+      </c>
+      <c r="E30" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B31" s="9">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="8">
+        <v>46302</v>
+      </c>
+      <c r="E31" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B32" s="9">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="8">
+        <v>46302</v>
+      </c>
+      <c r="E32" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B33" s="9">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" s="8">
+        <v>46302</v>
+      </c>
+      <c r="E33" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B34" s="9">
+        <v>3</v>
+      </c>
+      <c r="C34" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E34" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B35" s="9">
+        <v>3</v>
+      </c>
+      <c r="C35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E35" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B36" s="9">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>32</v>
+      </c>
+      <c r="D36" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E36" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B37" s="9">
+        <v>3</v>
+      </c>
+      <c r="C37" t="s">
+        <v>32</v>
+      </c>
+      <c r="D37" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E37" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B38" s="9">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>30</v>
+      </c>
+      <c r="D38" s="8">
+        <v>46308</v>
+      </c>
+      <c r="E38" t="s">
+        <v>40</v>
+      </c>
+      <c r="F38" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B39" s="9">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>30</v>
+      </c>
+      <c r="D39" s="8">
+        <v>46308</v>
+      </c>
+      <c r="E39" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B40" s="9">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>30</v>
+      </c>
+      <c r="D40" s="8">
+        <v>46308</v>
+      </c>
+      <c r="E40" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B41" s="9">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>30</v>
+      </c>
+      <c r="D41" s="8">
+        <v>46308</v>
+      </c>
+      <c r="E41" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B42" s="9">
+        <v>4</v>
+      </c>
+      <c r="C42" t="s">
+        <v>31</v>
+      </c>
+      <c r="D42" s="8">
+        <v>46309</v>
+      </c>
+      <c r="E42" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B43" s="9">
+        <v>4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>31</v>
+      </c>
+      <c r="D43" s="8">
+        <v>46309</v>
+      </c>
+      <c r="E43" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B44" s="9">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44" s="8">
+        <v>46309</v>
+      </c>
+      <c r="E44" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B45" s="9">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45" s="8">
+        <v>46309</v>
+      </c>
+      <c r="E45" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B46" s="9">
+        <v>4</v>
+      </c>
+      <c r="C46" t="s">
+        <v>32</v>
+      </c>
+      <c r="D46" s="8">
+        <v>46310</v>
+      </c>
+      <c r="E46" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B47" s="9">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>32</v>
+      </c>
+      <c r="D47" s="8">
+        <v>46310</v>
+      </c>
+      <c r="E47" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B48" s="9">
+        <v>4</v>
+      </c>
+      <c r="C48" t="s">
+        <v>32</v>
+      </c>
+      <c r="D48" s="8">
+        <v>46310</v>
+      </c>
+      <c r="E48" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B49" s="9">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>32</v>
+      </c>
+      <c r="D49" s="8">
+        <v>46310</v>
+      </c>
+      <c r="E49" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B50" s="9">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>30</v>
+      </c>
+      <c r="D50" s="8">
+        <v>46315</v>
+      </c>
+      <c r="E50" t="s">
+        <v>40</v>
+      </c>
+      <c r="F50" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B51" s="9">
+        <v>5</v>
+      </c>
+      <c r="C51" t="s">
+        <v>30</v>
+      </c>
+      <c r="D51" s="8">
+        <v>46315</v>
+      </c>
+      <c r="E51" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B52" s="9">
+        <v>5</v>
+      </c>
+      <c r="C52" t="s">
+        <v>30</v>
+      </c>
+      <c r="D52" s="8">
+        <v>46315</v>
+      </c>
+      <c r="E52" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B53" s="9">
+        <v>5</v>
+      </c>
+      <c r="C53" t="s">
+        <v>30</v>
+      </c>
+      <c r="D53" s="8">
+        <v>46315</v>
+      </c>
+      <c r="E53" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B54" s="9">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s">
+        <v>31</v>
+      </c>
+      <c r="D54" s="8">
+        <v>46316</v>
+      </c>
+      <c r="E54" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B55" s="9">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" s="8">
+        <v>46316</v>
+      </c>
+      <c r="E55" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B56" s="9">
+        <v>5</v>
+      </c>
+      <c r="C56" t="s">
+        <v>31</v>
+      </c>
+      <c r="D56" s="8">
+        <v>46316</v>
+      </c>
+      <c r="E56" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B57" s="9">
+        <v>5</v>
+      </c>
+      <c r="C57" t="s">
+        <v>31</v>
+      </c>
+      <c r="D57" s="8">
+        <v>46316</v>
+      </c>
+      <c r="E57" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B58" s="9">
+        <v>5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>32</v>
+      </c>
+      <c r="D58" s="8">
+        <v>46317</v>
+      </c>
+      <c r="E58" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B59" s="9">
+        <v>5</v>
+      </c>
+      <c r="C59" t="s">
+        <v>32</v>
+      </c>
+      <c r="D59" s="8">
+        <v>46317</v>
+      </c>
+      <c r="E59" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B60" s="9">
+        <v>5</v>
+      </c>
+      <c r="C60" t="s">
+        <v>32</v>
+      </c>
+      <c r="D60" s="8">
+        <v>46317</v>
+      </c>
+      <c r="E60" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B61" s="9">
+        <v>5</v>
+      </c>
+      <c r="C61" t="s">
+        <v>32</v>
+      </c>
+      <c r="D61" s="8">
+        <v>46317</v>
+      </c>
+      <c r="E61" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B62" s="9">
+        <v>6</v>
+      </c>
+      <c r="C62" t="s">
+        <v>30</v>
+      </c>
+      <c r="D62" s="8">
+        <v>46322</v>
+      </c>
+      <c r="E62" t="s">
+        <v>40</v>
+      </c>
+      <c r="F62" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B63" s="9">
+        <v>6</v>
+      </c>
+      <c r="C63" t="s">
+        <v>30</v>
+      </c>
+      <c r="D63" s="8">
+        <v>46322</v>
+      </c>
+      <c r="E63" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B64" s="9">
+        <v>6</v>
+      </c>
+      <c r="C64" t="s">
+        <v>30</v>
+      </c>
+      <c r="D64" s="8">
+        <v>46322</v>
+      </c>
+      <c r="E64" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B65" s="9">
+        <v>6</v>
+      </c>
+      <c r="C65" t="s">
+        <v>30</v>
+      </c>
+      <c r="D65" s="8">
+        <v>46322</v>
+      </c>
+      <c r="E65" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B66" s="9">
+        <v>6</v>
+      </c>
+      <c r="C66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D66" s="8">
+        <v>46323</v>
+      </c>
+      <c r="E66" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B67" s="9">
+        <v>6</v>
+      </c>
+      <c r="C67" t="s">
+        <v>31</v>
+      </c>
+      <c r="D67" s="8">
+        <v>46323</v>
+      </c>
+      <c r="E67" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B68" s="9">
+        <v>6</v>
+      </c>
+      <c r="C68" t="s">
+        <v>31</v>
+      </c>
+      <c r="D68" s="8">
+        <v>46323</v>
+      </c>
+      <c r="E68" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B69" s="9">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>31</v>
+      </c>
+      <c r="D69" s="8">
+        <v>46323</v>
+      </c>
+      <c r="E69" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B70" s="9">
+        <v>6</v>
+      </c>
+      <c r="C70" t="s">
+        <v>32</v>
+      </c>
+      <c r="D70" s="8">
+        <v>46324</v>
+      </c>
+      <c r="E70" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B71" s="9">
+        <v>6</v>
+      </c>
+      <c r="C71" t="s">
+        <v>32</v>
+      </c>
+      <c r="D71" s="8">
+        <v>46324</v>
+      </c>
+      <c r="E71" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B72" s="9">
+        <v>6</v>
+      </c>
+      <c r="C72" t="s">
+        <v>32</v>
+      </c>
+      <c r="D72" s="8">
+        <v>46324</v>
+      </c>
+      <c r="E72" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B73" s="9">
+        <v>6</v>
+      </c>
+      <c r="C73" t="s">
+        <v>32</v>
+      </c>
+      <c r="D73" s="8">
+        <v>46324</v>
+      </c>
+      <c r="E73" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B74" s="9">
+        <v>7</v>
+      </c>
+      <c r="C74" t="s">
+        <v>30</v>
+      </c>
+      <c r="D74" s="8">
+        <v>46329</v>
+      </c>
+      <c r="E74" t="s">
+        <v>40</v>
+      </c>
+      <c r="F74" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="75" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B75" s="9">
+        <v>7</v>
+      </c>
+      <c r="C75" t="s">
+        <v>30</v>
+      </c>
+      <c r="D75" s="8">
+        <v>46329</v>
+      </c>
+      <c r="E75" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B76" s="9">
+        <v>7</v>
+      </c>
+      <c r="C76" t="s">
+        <v>30</v>
+      </c>
+      <c r="D76" s="8">
+        <v>46329</v>
+      </c>
+      <c r="E76" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B77" s="9">
+        <v>7</v>
+      </c>
+      <c r="C77" t="s">
+        <v>30</v>
+      </c>
+      <c r="D77" s="8">
+        <v>46329</v>
+      </c>
+      <c r="E77" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B78" s="9">
+        <v>7</v>
+      </c>
+      <c r="C78" t="s">
+        <v>31</v>
+      </c>
+      <c r="D78" s="8">
+        <v>46330</v>
+      </c>
+      <c r="E78" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B79" s="9">
+        <v>7</v>
+      </c>
+      <c r="C79" t="s">
+        <v>31</v>
+      </c>
+      <c r="D79" s="8">
+        <v>46330</v>
+      </c>
+      <c r="E79" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B80" s="9">
+        <v>7</v>
+      </c>
+      <c r="C80" t="s">
+        <v>31</v>
+      </c>
+      <c r="D80" s="8">
+        <v>46330</v>
+      </c>
+      <c r="E80" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B81" s="9">
+        <v>7</v>
+      </c>
+      <c r="C81" t="s">
+        <v>31</v>
+      </c>
+      <c r="D81" s="8">
+        <v>46330</v>
+      </c>
+      <c r="E81" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="82" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B82" s="9">
+        <v>7</v>
+      </c>
+      <c r="C82" t="s">
+        <v>32</v>
+      </c>
+      <c r="D82" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E82" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="83" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B83" s="9">
+        <v>7</v>
+      </c>
+      <c r="C83" t="s">
+        <v>32</v>
+      </c>
+      <c r="D83" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E83" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B84" s="9">
+        <v>7</v>
+      </c>
+      <c r="C84" t="s">
+        <v>32</v>
+      </c>
+      <c r="D84" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E84" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="85" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B85" s="9">
+        <v>7</v>
+      </c>
+      <c r="C85" t="s">
+        <v>32</v>
+      </c>
+      <c r="D85" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E85" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bug fix points calc
</commit_message>
<xml_diff>
--- a/database/series_setup.xlsx
+++ b/database/series_setup.xlsx
@@ -4,19 +4,20 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
     <sheet name="Stages" sheetId="2" r:id="rId2"/>
     <sheet name="Races" sheetId="3" r:id="rId3"/>
+    <sheet name="community" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="89">
   <si>
     <t>Name</t>
   </si>
@@ -274,6 +275,15 @@
   </si>
   <si>
     <t>95da701b-925e-4601-8001-2440e419b211</t>
+  </si>
+  <si>
+    <t>52298c21-d570-4e4c-b162-997822baef64</t>
+  </si>
+  <si>
+    <t>49ebc53c-910a-45f9-b3ff-8fe8587b1a5a</t>
+  </si>
+  <si>
+    <t>https://riders.rouvy.com/social/communities/bf28346e-e6fc-4e35-b7d4-0a43b950c96a</t>
   </si>
 </sst>
 </file>
@@ -929,7 +939,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.77734375" bestFit="1" customWidth="1"/>
@@ -1492,24 +1502,24 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="B33" s="9">
         <v>3</v>
       </c>
       <c r="C33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D33" s="8">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E33" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B34" s="9">
         <v>3</v>
@@ -1521,12 +1531,12 @@
         <v>46302</v>
       </c>
       <c r="E34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B35" s="9">
         <v>3</v>
@@ -1538,12 +1548,12 @@
         <v>46302</v>
       </c>
       <c r="E35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B36" s="9">
         <v>3</v>
@@ -1555,29 +1565,29 @@
         <v>46302</v>
       </c>
       <c r="E36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B37" s="9">
         <v>3</v>
       </c>
       <c r="C37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D37" s="8">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E37" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B38" s="9">
         <v>3</v>
@@ -1589,12 +1599,12 @@
         <v>46303</v>
       </c>
       <c r="E38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B39" s="9">
         <v>3</v>
@@ -1606,12 +1616,12 @@
         <v>46303</v>
       </c>
       <c r="E39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B40" s="9">
         <v>3</v>
@@ -1623,38 +1633,41 @@
         <v>46303</v>
       </c>
       <c r="E40" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="9">
+        <v>3</v>
+      </c>
+      <c r="C41" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E41" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B41" s="9">
-        <v>4</v>
-      </c>
-      <c r="C41" t="s">
-        <v>29</v>
-      </c>
-      <c r="D41" s="8">
-        <v>46308</v>
-      </c>
-      <c r="E41" t="s">
-        <v>33</v>
-      </c>
-      <c r="F41" t="s">
-        <v>40</v>
-      </c>
-    </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>87</v>
+      </c>
       <c r="B42" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D42" s="8">
-        <v>46308</v>
+        <v>46303</v>
       </c>
       <c r="E42" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1668,7 +1681,10 @@
         <v>46308</v>
       </c>
       <c r="E43" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="F43" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1682,7 +1698,7 @@
         <v>46308</v>
       </c>
       <c r="E44" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1690,13 +1706,13 @@
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D45" s="8">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E45" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1704,13 +1720,13 @@
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D46" s="8">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E46" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1724,7 +1740,7 @@
         <v>46309</v>
       </c>
       <c r="E47" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1738,7 +1754,7 @@
         <v>46309</v>
       </c>
       <c r="E48" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.3">
@@ -1746,13 +1762,13 @@
         <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D49" s="8">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E49" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="50" spans="2:6" x14ac:dyDescent="0.3">
@@ -1760,13 +1776,13 @@
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D50" s="8">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E50" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.3">
@@ -1780,7 +1796,7 @@
         <v>46310</v>
       </c>
       <c r="E51" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.3">
@@ -1794,38 +1810,35 @@
         <v>46310</v>
       </c>
       <c r="E52" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D53" s="8">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="E53" t="s">
-        <v>33</v>
-      </c>
-      <c r="F53" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D54" s="8">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="E54" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.3">
@@ -1839,7 +1852,10 @@
         <v>46315</v>
       </c>
       <c r="E55" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="F55" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.3">
@@ -1853,7 +1869,7 @@
         <v>46315</v>
       </c>
       <c r="E56" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.3">
@@ -1861,13 +1877,13 @@
         <v>5</v>
       </c>
       <c r="C57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D57" s="8">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="E57" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.3">
@@ -1875,13 +1891,13 @@
         <v>5</v>
       </c>
       <c r="C58" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D58" s="8">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="E58" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.3">
@@ -1895,7 +1911,7 @@
         <v>46316</v>
       </c>
       <c r="E59" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.3">
@@ -1909,7 +1925,7 @@
         <v>46316</v>
       </c>
       <c r="E60" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.3">
@@ -1917,13 +1933,13 @@
         <v>5</v>
       </c>
       <c r="C61" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D61" s="8">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="E61" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.3">
@@ -1931,13 +1947,13 @@
         <v>5</v>
       </c>
       <c r="C62" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D62" s="8">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="E62" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.3">
@@ -1951,7 +1967,7 @@
         <v>46317</v>
       </c>
       <c r="E63" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.3">
@@ -1965,38 +1981,35 @@
         <v>46317</v>
       </c>
       <c r="E64" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B65" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C65" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D65" s="8">
-        <v>46322</v>
+        <v>46317</v>
       </c>
       <c r="E65" t="s">
-        <v>33</v>
-      </c>
-      <c r="F65" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B66" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C66" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D66" s="8">
-        <v>46322</v>
+        <v>46317</v>
       </c>
       <c r="E66" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.3">
@@ -2010,7 +2023,10 @@
         <v>46322</v>
       </c>
       <c r="E67" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="F67" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.3">
@@ -2024,7 +2040,7 @@
         <v>46322</v>
       </c>
       <c r="E68" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.3">
@@ -2032,13 +2048,13 @@
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D69" s="8">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="E69" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.3">
@@ -2046,13 +2062,13 @@
         <v>6</v>
       </c>
       <c r="C70" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D70" s="8">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="E70" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.3">
@@ -2066,7 +2082,7 @@
         <v>46323</v>
       </c>
       <c r="E71" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.3">
@@ -2080,7 +2096,7 @@
         <v>46323</v>
       </c>
       <c r="E72" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.3">
@@ -2088,13 +2104,13 @@
         <v>6</v>
       </c>
       <c r="C73" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D73" s="8">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="E73" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.3">
@@ -2102,13 +2118,13 @@
         <v>6</v>
       </c>
       <c r="C74" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D74" s="8">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="E74" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="75" spans="2:6" x14ac:dyDescent="0.3">
@@ -2122,7 +2138,7 @@
         <v>46324</v>
       </c>
       <c r="E75" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.3">
@@ -2136,38 +2152,35 @@
         <v>46324</v>
       </c>
       <c r="E76" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C77" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D77" s="8">
-        <v>46329</v>
+        <v>46324</v>
       </c>
       <c r="E77" t="s">
-        <v>33</v>
-      </c>
-      <c r="F77" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C78" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D78" s="8">
-        <v>46329</v>
+        <v>46324</v>
       </c>
       <c r="E78" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="79" spans="2:6" x14ac:dyDescent="0.3">
@@ -2181,7 +2194,10 @@
         <v>46329</v>
       </c>
       <c r="E79" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="F79" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="80" spans="2:6" x14ac:dyDescent="0.3">
@@ -2195,7 +2211,7 @@
         <v>46329</v>
       </c>
       <c r="E80" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.3">
@@ -2203,13 +2219,13 @@
         <v>7</v>
       </c>
       <c r="C81" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D81" s="8">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="E81" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.3">
@@ -2217,13 +2233,13 @@
         <v>7</v>
       </c>
       <c r="C82" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D82" s="8">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="E82" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.3">
@@ -2237,7 +2253,7 @@
         <v>46330</v>
       </c>
       <c r="E83" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.3">
@@ -2251,7 +2267,7 @@
         <v>46330</v>
       </c>
       <c r="E84" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.3">
@@ -2259,13 +2275,13 @@
         <v>7</v>
       </c>
       <c r="C85" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D85" s="8">
-        <v>46331</v>
+        <v>46330</v>
       </c>
       <c r="E85" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.3">
@@ -2273,13 +2289,13 @@
         <v>7</v>
       </c>
       <c r="C86" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D86" s="8">
-        <v>46331</v>
+        <v>46330</v>
       </c>
       <c r="E86" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.3">
@@ -2293,7 +2309,7 @@
         <v>46331</v>
       </c>
       <c r="E87" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.3">
@@ -2307,7 +2323,50 @@
         <v>46331</v>
       </c>
       <c r="E88" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B89" s="9">
+        <v>7</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E89" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B90" s="9">
+        <v>7</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E90" t="s">
         <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="3" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added Stage 4 races
</commit_message>
<xml_diff>
--- a/database/series_setup.xlsx
+++ b/database/series_setup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="3"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="103">
   <si>
     <t>Name</t>
   </si>
@@ -284,6 +284,48 @@
   </si>
   <si>
     <t>https://riders.rouvy.com/social/communities/bf28346e-e6fc-4e35-b7d4-0a43b950c96a</t>
+  </si>
+  <si>
+    <t>aac27817-4819-45df-8c79-da1d0f04e9ad</t>
+  </si>
+  <si>
+    <t>637cc281-19b0-48d1-8eb6-f54f95ddc552</t>
+  </si>
+  <si>
+    <t>7de00311-672a-433e-a3f7-8d2b8ae45919</t>
+  </si>
+  <si>
+    <t>e49abcf8-6074-448c-b530-fa68f8b64cd1</t>
+  </si>
+  <si>
+    <t>522a182b-861b-4070-8665-8a8f07349dc9</t>
+  </si>
+  <si>
+    <t>6396cbd4-d81e-43ff-9638-5a54f30af79c</t>
+  </si>
+  <si>
+    <t>af71abb5-3610-4185-a5e8-4d3ab0b60081</t>
+  </si>
+  <si>
+    <t>f67bd35a-9d1c-41ff-a404-d5e78c09f1de</t>
+  </si>
+  <si>
+    <t>22e8bfd3-2b83-4f40-acec-4c57dbb5af8c</t>
+  </si>
+  <si>
+    <t>bf89e7be-b231-472b-bda9-1c90e8373b48</t>
+  </si>
+  <si>
+    <t>f666b64b-5c9d-46ab-b9bf-7da95b39ed79</t>
+  </si>
+  <si>
+    <t>c4434133-dbd8-485c-8b7c-d9f99f7a89ae</t>
+  </si>
+  <si>
+    <t>2a90861b-95d8-465d-aa68-ffba2f353260</t>
+  </si>
+  <si>
+    <t>80ea2193-0429-4b57-b71e-e8e78f424926</t>
   </si>
 </sst>
 </file>
@@ -939,7 +981,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.77734375" bestFit="1" customWidth="1"/>
@@ -1671,6 +1713,9 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>89</v>
+      </c>
       <c r="B43" s="9">
         <v>4</v>
       </c>
@@ -1688,6 +1733,9 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>90</v>
+      </c>
       <c r="B44" s="9">
         <v>4</v>
       </c>
@@ -1702,6 +1750,9 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>91</v>
+      </c>
       <c r="B45" s="9">
         <v>4</v>
       </c>
@@ -1716,6 +1767,9 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>92</v>
+      </c>
       <c r="B46" s="9">
         <v>4</v>
       </c>
@@ -1730,20 +1784,26 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>93</v>
+      </c>
       <c r="B47" s="9">
         <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D47" s="8">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="E47" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>94</v>
+      </c>
       <c r="B48" s="9">
         <v>4</v>
       </c>
@@ -1754,10 +1814,13 @@
         <v>46309</v>
       </c>
       <c r="E48" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>95</v>
+      </c>
       <c r="B49" s="9">
         <v>4</v>
       </c>
@@ -1768,10 +1831,13 @@
         <v>46309</v>
       </c>
       <c r="E49" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>96</v>
+      </c>
       <c r="B50" s="9">
         <v>4</v>
       </c>
@@ -1782,24 +1848,30 @@
         <v>46309</v>
       </c>
       <c r="E50" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>97</v>
+      </c>
       <c r="B51" s="9">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D51" s="8">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="E51" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>98</v>
+      </c>
       <c r="B52" s="9">
         <v>4</v>
       </c>
@@ -1810,10 +1882,13 @@
         <v>46310</v>
       </c>
       <c r="E52" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>99</v>
+      </c>
       <c r="B53" s="9">
         <v>4</v>
       </c>
@@ -1824,10 +1899,13 @@
         <v>46310</v>
       </c>
       <c r="E53" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>100</v>
+      </c>
       <c r="B54" s="9">
         <v>4</v>
       </c>
@@ -1838,41 +1916,44 @@
         <v>46310</v>
       </c>
       <c r="E54" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>101</v>
+      </c>
+      <c r="B55" s="9">
+        <v>4</v>
+      </c>
+      <c r="C55" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" s="8">
+        <v>46310</v>
+      </c>
+      <c r="E55" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B55" s="9">
-        <v>5</v>
-      </c>
-      <c r="C55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D55" s="8">
-        <v>46315</v>
-      </c>
-      <c r="E55" t="s">
-        <v>33</v>
-      </c>
-      <c r="F55" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>102</v>
+      </c>
       <c r="B56" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D56" s="8">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="E56" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B57" s="9">
         <v>5</v>
       </c>
@@ -1883,10 +1964,13 @@
         <v>46315</v>
       </c>
       <c r="E57" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="F57" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B58" s="9">
         <v>5</v>
       </c>
@@ -1897,38 +1981,38 @@
         <v>46315</v>
       </c>
       <c r="E58" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B59" s="9">
         <v>5</v>
       </c>
       <c r="C59" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D59" s="8">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="E59" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B60" s="9">
         <v>5</v>
       </c>
       <c r="C60" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D60" s="8">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="E60" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B61" s="9">
         <v>5</v>
       </c>
@@ -1939,10 +2023,10 @@
         <v>46316</v>
       </c>
       <c r="E61" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B62" s="9">
         <v>5</v>
       </c>
@@ -1953,35 +2037,35 @@
         <v>46316</v>
       </c>
       <c r="E62" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B63" s="9">
         <v>5</v>
       </c>
       <c r="C63" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D63" s="8">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="E63" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B64" s="9">
         <v>5</v>
       </c>
       <c r="C64" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D64" s="8">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="E64" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.3">
@@ -1995,7 +2079,7 @@
         <v>46317</v>
       </c>
       <c r="E65" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.3">
@@ -2009,38 +2093,35 @@
         <v>46317</v>
       </c>
       <c r="E66" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B67" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C67" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D67" s="8">
-        <v>46322</v>
+        <v>46317</v>
       </c>
       <c r="E67" t="s">
-        <v>33</v>
-      </c>
-      <c r="F67" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B68" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C68" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D68" s="8">
-        <v>46322</v>
+        <v>46317</v>
       </c>
       <c r="E68" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.3">
@@ -2054,7 +2135,10 @@
         <v>46322</v>
       </c>
       <c r="E69" t="s">
-        <v>35</v>
+        <v>33</v>
+      </c>
+      <c r="F69" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.3">
@@ -2068,7 +2152,7 @@
         <v>46322</v>
       </c>
       <c r="E70" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.3">
@@ -2076,13 +2160,13 @@
         <v>6</v>
       </c>
       <c r="C71" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D71" s="8">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="E71" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.3">
@@ -2090,13 +2174,13 @@
         <v>6</v>
       </c>
       <c r="C72" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D72" s="8">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="E72" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.3">
@@ -2110,7 +2194,7 @@
         <v>46323</v>
       </c>
       <c r="E73" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.3">
@@ -2124,7 +2208,7 @@
         <v>46323</v>
       </c>
       <c r="E74" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="75" spans="2:6" x14ac:dyDescent="0.3">
@@ -2132,13 +2216,13 @@
         <v>6</v>
       </c>
       <c r="C75" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D75" s="8">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="E75" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.3">
@@ -2146,13 +2230,13 @@
         <v>6</v>
       </c>
       <c r="C76" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D76" s="8">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="E76" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.3">
@@ -2166,7 +2250,7 @@
         <v>46324</v>
       </c>
       <c r="E77" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="78" spans="2:6" x14ac:dyDescent="0.3">
@@ -2180,41 +2264,38 @@
         <v>46324</v>
       </c>
       <c r="E78" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C79" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D79" s="8">
-        <v>46329</v>
+        <v>46324</v>
       </c>
       <c r="E79" t="s">
-        <v>33</v>
-      </c>
-      <c r="F79" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C80" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D80" s="8">
-        <v>46329</v>
+        <v>46324</v>
       </c>
       <c r="E80" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="9">
         <v>7</v>
       </c>
@@ -2225,10 +2306,13 @@
         <v>46329</v>
       </c>
       <c r="E81" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="F81" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="9">
         <v>7</v>
       </c>
@@ -2239,38 +2323,38 @@
         <v>46329</v>
       </c>
       <c r="E82" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="9">
         <v>7</v>
       </c>
       <c r="C83" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D83" s="8">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="E83" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="84" spans="2:5" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="9">
         <v>7</v>
       </c>
       <c r="C84" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D84" s="8">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="E84" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="85" spans="2:5" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="9">
         <v>7</v>
       </c>
@@ -2281,10 +2365,10 @@
         <v>46330</v>
       </c>
       <c r="E85" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="86" spans="2:5" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="9">
         <v>7</v>
       </c>
@@ -2295,38 +2379,38 @@
         <v>46330</v>
       </c>
       <c r="E86" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="9">
         <v>7</v>
       </c>
       <c r="C87" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D87" s="8">
-        <v>46331</v>
+        <v>46330</v>
       </c>
       <c r="E87" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="9">
         <v>7</v>
       </c>
       <c r="C88" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D88" s="8">
-        <v>46331</v>
+        <v>46330</v>
       </c>
       <c r="E88" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="89" spans="2:5" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="9">
         <v>7</v>
       </c>
@@ -2337,10 +2421,10 @@
         <v>46331</v>
       </c>
       <c r="E89" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="9">
         <v>7</v>
       </c>
@@ -2351,6 +2435,34 @@
         <v>46331</v>
       </c>
       <c r="E90" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B91" s="9">
+        <v>7</v>
+      </c>
+      <c r="C91" t="s">
+        <v>31</v>
+      </c>
+      <c r="D91" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E91" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B92" s="9">
+        <v>7</v>
+      </c>
+      <c r="C92" t="s">
+        <v>31</v>
+      </c>
+      <c r="D92" s="8">
+        <v>46331</v>
+      </c>
+      <c r="E92" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>